<commit_message>
feat: Add extended German medal showcase for Grand Cross and Star of Grand Cross
Add germany_ext coordinate section (grand_cross_big1, star_grand_cross_big1)
to the career award coordinates JSON. Detection checks for achievement folders
201037/201038 under game_dir at request time; falls back gracefully to the
standard germany layout when absent. i18n keys and narratives added in all
7 locales.
</commit_message>
<xml_diff>
--- a/IL-2_Tracker_career_award_coordinates.xlsx
+++ b/IL-2_Tracker_career_award_coordinates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bleih\source\repos\IL-2-Campaign-Tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB5B9B03-9396-48AA-BF9A-41EA30651720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFEC9439-3FB8-4B05-A9ED-166307EDDAED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14844" yWindow="1380" windowWidth="29508" windowHeight="23784" xr2:uid="{E6D131E9-51AD-48C7-A8DF-61BD79F7615F}"/>
+    <workbookView xWindow="32796" yWindow="1296" windowWidth="25296" windowHeight="23784" xr2:uid="{E6D131E9-51AD-48C7-A8DF-61BD79F7615F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="125">
   <si>
     <t>USSR (early)</t>
   </si>
@@ -402,6 +402,15 @@
   </si>
   <si>
     <t>DSM_big1</t>
+  </si>
+  <si>
+    <t>grand_cross_big1</t>
+  </si>
+  <si>
+    <t>star_grand_cross_big1</t>
+  </si>
+  <si>
+    <t>Germany_overlay_ext</t>
   </si>
 </sst>
 </file>
@@ -776,7 +785,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B16B5802-CA93-448F-941A-C8431B7D54EA}">
-  <dimension ref="A1:Y77"/>
+  <dimension ref="A1:Y80"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.21875" customWidth="1"/>
@@ -1992,267 +2001,318 @@
     </row>
     <row r="64" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>67</v>
+        <v>122</v>
       </c>
       <c r="B64">
-        <v>32</v>
+        <v>1978</v>
       </c>
       <c r="C64">
-        <v>0</v>
+        <v>125</v>
       </c>
       <c r="D64">
-        <v>2018</v>
+        <v>461</v>
       </c>
       <c r="E64">
-        <v>961</v>
+        <v>512</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>123</v>
+      </c>
+      <c r="B65">
+        <v>1978</v>
+      </c>
+      <c r="C65">
+        <v>661</v>
+      </c>
+      <c r="D65">
+        <v>460</v>
+      </c>
+      <c r="E65">
+        <v>458</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>69</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C66" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E66" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G66" s="1" t="s">
-        <v>17</v>
+        <v>67</v>
+      </c>
+      <c r="B66">
+        <v>32</v>
+      </c>
+      <c r="C66">
+        <v>0</v>
+      </c>
+      <c r="D66">
+        <v>2018</v>
+      </c>
+      <c r="E66">
+        <v>961</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>70</v>
+        <v>124</v>
       </c>
       <c r="B67">
-        <v>178</v>
+        <v>0</v>
       </c>
       <c r="C67">
-        <v>141</v>
+        <v>79</v>
       </c>
       <c r="D67">
-        <v>258</v>
+        <v>2481</v>
       </c>
       <c r="E67">
-        <v>494</v>
-      </c>
-      <c r="G67" t="s">
-        <v>71</v>
-      </c>
-      <c r="H67" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A68" t="s">
-        <v>73</v>
-      </c>
-      <c r="B68">
-        <v>513</v>
-      </c>
-      <c r="C68">
-        <v>141</v>
-      </c>
-      <c r="D68">
-        <v>302</v>
-      </c>
-      <c r="E68">
-        <v>493</v>
-      </c>
-      <c r="G68" t="s">
-        <v>74</v>
-      </c>
-      <c r="H68" t="s">
-        <v>75</v>
+        <v>967</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>76</v>
-      </c>
-      <c r="B69">
-        <v>881</v>
-      </c>
-      <c r="C69">
-        <v>180</v>
-      </c>
-      <c r="D69">
-        <v>288</v>
-      </c>
-      <c r="E69">
-        <v>504</v>
-      </c>
-      <c r="G69" t="s">
-        <v>77</v>
+        <v>69</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="B70">
-        <v>1257</v>
+        <v>178</v>
       </c>
       <c r="C70">
         <v>141</v>
       </c>
       <c r="D70">
-        <v>280</v>
+        <v>258</v>
       </c>
       <c r="E70">
-        <v>498</v>
+        <v>494</v>
       </c>
       <c r="G70" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="H70" t="s">
-        <v>80</v>
-      </c>
-      <c r="I70" t="s">
-        <v>96</v>
+        <v>72</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="B71">
-        <v>1614</v>
+        <v>513</v>
       </c>
       <c r="C71">
         <v>141</v>
       </c>
       <c r="D71">
-        <v>258</v>
+        <v>302</v>
       </c>
       <c r="E71">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="G71" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="H71" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="B72">
-        <v>1087</v>
+        <v>881</v>
       </c>
       <c r="C72">
-        <v>639</v>
+        <v>180</v>
       </c>
       <c r="D72">
-        <v>471</v>
+        <v>288</v>
       </c>
       <c r="E72">
-        <v>265</v>
+        <v>504</v>
+      </c>
+      <c r="G72" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B73">
-        <v>580</v>
+        <v>1257</v>
       </c>
       <c r="C73">
-        <v>657</v>
+        <v>141</v>
       </c>
       <c r="D73">
-        <v>470</v>
+        <v>280</v>
       </c>
       <c r="E73">
-        <v>500</v>
+        <v>498</v>
+      </c>
+      <c r="G73" t="s">
+        <v>79</v>
+      </c>
+      <c r="H73" t="s">
+        <v>80</v>
+      </c>
+      <c r="I73" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B74">
-        <v>1073</v>
+        <v>1614</v>
       </c>
       <c r="C74">
-        <v>861</v>
+        <v>141</v>
       </c>
       <c r="D74">
-        <v>502</v>
+        <v>258</v>
       </c>
       <c r="E74">
-        <v>284</v>
+        <v>494</v>
       </c>
       <c r="G74" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="H74" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B75">
-        <v>1597</v>
+        <v>1087</v>
       </c>
       <c r="C75">
-        <v>648</v>
+        <v>639</v>
       </c>
       <c r="D75">
-        <v>293</v>
+        <v>471</v>
       </c>
       <c r="E75">
-        <v>497</v>
-      </c>
-      <c r="G75" t="s">
-        <v>90</v>
-      </c>
-      <c r="H75" t="s">
-        <v>91</v>
+        <v>265</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B76">
-        <v>158</v>
+        <v>580</v>
       </c>
       <c r="C76">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="D76">
-        <v>299</v>
+        <v>470</v>
       </c>
       <c r="E76">
-        <v>486</v>
+        <v>500</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
+        <v>86</v>
+      </c>
+      <c r="B77">
+        <v>1073</v>
+      </c>
+      <c r="C77">
+        <v>861</v>
+      </c>
+      <c r="D77">
+        <v>502</v>
+      </c>
+      <c r="E77">
+        <v>284</v>
+      </c>
+      <c r="G77" t="s">
+        <v>87</v>
+      </c>
+      <c r="H77" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>89</v>
+      </c>
+      <c r="B78">
+        <v>1597</v>
+      </c>
+      <c r="C78">
+        <v>648</v>
+      </c>
+      <c r="D78">
+        <v>293</v>
+      </c>
+      <c r="E78">
+        <v>497</v>
+      </c>
+      <c r="G78" t="s">
+        <v>90</v>
+      </c>
+      <c r="H78" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>93</v>
+      </c>
+      <c r="B79">
+        <v>158</v>
+      </c>
+      <c r="C79">
+        <v>654</v>
+      </c>
+      <c r="D79">
+        <v>299</v>
+      </c>
+      <c r="E79">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
         <v>92</v>
       </c>
-      <c r="B77">
+      <c r="B80">
         <v>32</v>
       </c>
-      <c r="C77">
+      <c r="C80">
         <v>0</v>
       </c>
-      <c r="D77">
+      <c r="D80">
         <v>2018</v>
       </c>
-      <c r="E77">
+      <c r="E80">
         <v>961</v>
       </c>
     </row>

</xml_diff>